<commit_message>
Gesi added to the map
</commit_message>
<xml_diff>
--- a/public/EI VI MPI with components.xlsx
+++ b/public/EI VI MPI with components.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work - IES\Shared Prosperity Mapping\Analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7207455-601C-4B2C-B20F-BB403FC796FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4977168E-5B9A-473C-917B-F33B82DBED46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,15 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -87,9 +96,6 @@
     <t>Gadhi</t>
   </si>
   <si>
-    <t>Kepilasgadhi</t>
-  </si>
-  <si>
     <t>Sunkoshi</t>
   </si>
   <si>
@@ -123,13 +129,16 @@
     <t>Contribution % 3.6</t>
   </si>
   <si>
-    <t>Halesi</t>
+    <t>MPI%</t>
   </si>
   <si>
-    <t>Hanumanangar</t>
+    <t>Kepilasagadhi</t>
   </si>
   <si>
-    <t>MPI%</t>
+    <t>Halesi Tuwachung</t>
+  </si>
+  <si>
+    <t>Hanumannagar Kankalani</t>
   </si>
 </sst>
 </file>
@@ -231,7 +240,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -256,13 +265,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,8 +558,8 @@
     <col min="10" max="19" width="16.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" style="12" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" style="16" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10" style="16" customWidth="1"/>
+    <col min="22" max="22" width="10" style="12" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10" style="12" customWidth="1"/>
     <col min="24" max="26" width="12" style="3" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="12" style="12" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="12.44140625" style="12" customWidth="1"/>
@@ -592,34 +595,34 @@
         <v>7</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="T1" s="9" t="s">
         <v>8</v>
@@ -627,11 +630,11 @@
       <c r="U1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="V1" s="14" t="s">
+      <c r="V1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="W1" s="14" t="s">
-        <v>34</v>
+      <c r="W1" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>11</v>
@@ -654,7 +657,7 @@
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
@@ -716,10 +719,10 @@
       <c r="U2" s="8">
         <v>0.3710317460317461</v>
       </c>
-      <c r="V2" s="15">
+      <c r="V2" s="14">
         <v>0.15505804311774499</v>
       </c>
-      <c r="W2" s="15">
+      <c r="W2" s="14">
         <f>V2*100</f>
         <v>15.505804311774499</v>
       </c>
@@ -745,7 +748,7 @@
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
@@ -807,10 +810,10 @@
       <c r="U3" s="8">
         <v>0.39285714285714279</v>
       </c>
-      <c r="V3" s="15">
+      <c r="V3" s="14">
         <v>0.14864864864864863</v>
       </c>
-      <c r="W3" s="15">
+      <c r="W3" s="14">
         <f t="shared" ref="W3:W55" si="0">V3*100</f>
         <v>14.864864864864863</v>
       </c>
@@ -836,7 +839,7 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
@@ -898,10 +901,10 @@
       <c r="U4" s="8">
         <v>0.40972222222222227</v>
       </c>
-      <c r="V4" s="15">
+      <c r="V4" s="14">
         <v>7.9945799457994585E-2</v>
       </c>
-      <c r="W4" s="15">
+      <c r="W4" s="14">
         <f t="shared" si="0"/>
         <v>7.9945799457994582</v>
       </c>
@@ -927,7 +930,7 @@
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B5" s="7">
         <v>4</v>
@@ -989,10 +992,10 @@
       <c r="U5" s="8">
         <v>0.37901234567901254</v>
       </c>
-      <c r="V5" s="15">
+      <c r="V5" s="14">
         <v>0.19163545568039961</v>
       </c>
-      <c r="W5" s="15">
+      <c r="W5" s="14">
         <f t="shared" si="0"/>
         <v>19.163545568039961</v>
       </c>
@@ -1018,7 +1021,7 @@
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B6" s="7">
         <v>5</v>
@@ -1080,10 +1083,10 @@
       <c r="U6" s="8">
         <v>0.39130434782608703</v>
       </c>
-      <c r="V6" s="15">
+      <c r="V6" s="14">
         <v>0.15000000000000005</v>
       </c>
-      <c r="W6" s="15">
+      <c r="W6" s="14">
         <f t="shared" si="0"/>
         <v>15.000000000000005</v>
       </c>
@@ -1109,7 +1112,7 @@
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B7" s="7">
         <v>6</v>
@@ -1171,10 +1174,10 @@
       <c r="U7" s="8">
         <v>0.4494949494949495</v>
       </c>
-      <c r="V7" s="15">
+      <c r="V7" s="14">
         <v>0.26023391812865498</v>
       </c>
-      <c r="W7" s="15">
+      <c r="W7" s="14">
         <f t="shared" si="0"/>
         <v>26.023391812865498</v>
       </c>
@@ -1200,7 +1203,7 @@
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B8" s="7">
         <v>7</v>
@@ -1262,10 +1265,10 @@
       <c r="U8" s="8">
         <v>0.43548387096774205</v>
       </c>
-      <c r="V8" s="15">
+      <c r="V8" s="14">
         <v>0.22131147540983612</v>
       </c>
-      <c r="W8" s="15">
+      <c r="W8" s="14">
         <f t="shared" si="0"/>
         <v>22.131147540983612</v>
       </c>
@@ -1291,7 +1294,7 @@
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="7">
         <v>1</v>
@@ -1353,10 +1356,10 @@
       <c r="U9" s="8">
         <v>0.37111111111111117</v>
       </c>
-      <c r="V9" s="15">
+      <c r="V9" s="14">
         <v>0.17505241090146753</v>
       </c>
-      <c r="W9" s="15">
+      <c r="W9" s="14">
         <f t="shared" si="0"/>
         <v>17.505241090146754</v>
       </c>
@@ -1382,7 +1385,7 @@
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" s="7">
         <v>2</v>
@@ -1444,10 +1447,10 @@
       <c r="U10" s="8">
         <v>0.35069444444444448</v>
       </c>
-      <c r="V10" s="15">
+      <c r="V10" s="14">
         <v>9.67432950191571E-2</v>
       </c>
-      <c r="W10" s="15">
+      <c r="W10" s="14">
         <f t="shared" si="0"/>
         <v>9.6743295019157092</v>
       </c>
@@ -1473,7 +1476,7 @@
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="7">
         <v>3</v>
@@ -1535,10 +1538,10 @@
       <c r="U11" s="8">
         <v>0.39506172839506193</v>
       </c>
-      <c r="V11" s="15">
+      <c r="V11" s="14">
         <v>0.24521072796934879</v>
       </c>
-      <c r="W11" s="15">
+      <c r="W11" s="14">
         <f t="shared" si="0"/>
         <v>24.521072796934877</v>
       </c>
@@ -1564,7 +1567,7 @@
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="7">
         <v>4</v>
@@ -1626,10 +1629,10 @@
       <c r="U12" s="8">
         <v>0.34722222222222232</v>
       </c>
-      <c r="V12" s="15">
+      <c r="V12" s="14">
         <v>5.3418803418803437E-2</v>
       </c>
-      <c r="W12" s="15">
+      <c r="W12" s="14">
         <f t="shared" si="0"/>
         <v>5.3418803418803433</v>
       </c>
@@ -1655,7 +1658,7 @@
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13" s="7">
         <v>5</v>
@@ -1717,10 +1720,10 @@
       <c r="U13" s="8">
         <v>0.3541666666666668</v>
       </c>
-      <c r="V13" s="15">
+      <c r="V13" s="14">
         <v>4.2288557213930364E-2</v>
       </c>
-      <c r="W13" s="15">
+      <c r="W13" s="14">
         <f t="shared" si="0"/>
         <v>4.2288557213930362</v>
       </c>
@@ -1746,7 +1749,7 @@
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="7">
         <v>6</v>
@@ -1808,10 +1811,10 @@
       <c r="U14" s="8">
         <v>0.36111111111111116</v>
       </c>
-      <c r="V14" s="15">
+      <c r="V14" s="14">
         <v>1.8055555555555557E-2</v>
       </c>
-      <c r="W14" s="15">
+      <c r="W14" s="14">
         <f t="shared" si="0"/>
         <v>1.8055555555555558</v>
       </c>
@@ -1837,7 +1840,7 @@
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="7">
         <v>7</v>
@@ -1899,10 +1902,10 @@
       <c r="U15" s="8">
         <v>0.3492063492063493</v>
       </c>
-      <c r="V15" s="15">
+      <c r="V15" s="14">
         <v>4.0072859744990905E-2</v>
       </c>
-      <c r="W15" s="15">
+      <c r="W15" s="14">
         <f t="shared" si="0"/>
         <v>4.0072859744990907</v>
       </c>
@@ -1928,7 +1931,7 @@
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="7">
         <v>8</v>
@@ -1990,10 +1993,10 @@
       <c r="U16" s="8">
         <v>0.35416666666666669</v>
       </c>
-      <c r="V16" s="15">
+      <c r="V16" s="14">
         <v>0.13492063492063491</v>
       </c>
-      <c r="W16" s="15">
+      <c r="W16" s="14">
         <f t="shared" si="0"/>
         <v>13.492063492063492</v>
       </c>
@@ -2019,7 +2022,7 @@
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17" s="7">
         <v>9</v>
@@ -2081,10 +2084,10 @@
       <c r="U17" s="8">
         <v>0.33333333333333343</v>
       </c>
-      <c r="V17" s="15">
+      <c r="V17" s="14">
         <v>9.7222222222222252E-2</v>
       </c>
-      <c r="W17" s="15">
+      <c r="W17" s="14">
         <f t="shared" si="0"/>
         <v>9.722222222222225</v>
       </c>
@@ -2110,7 +2113,7 @@
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B18" s="7">
         <v>10</v>
@@ -2172,10 +2175,10 @@
       <c r="U18" s="8">
         <v>0.34362139917695472</v>
       </c>
-      <c r="V18" s="15">
+      <c r="V18" s="14">
         <v>0.16868686868686869</v>
       </c>
-      <c r="W18" s="15">
+      <c r="W18" s="14">
         <f t="shared" si="0"/>
         <v>16.868686868686869</v>
       </c>
@@ -2201,7 +2204,7 @@
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" s="7">
         <v>11</v>
@@ -2263,10 +2266,10 @@
       <c r="U19" s="8">
         <v>0.35353535353535359</v>
       </c>
-      <c r="V19" s="15">
+      <c r="V19" s="14">
         <v>7.3375262054507354E-2</v>
       </c>
-      <c r="W19" s="15">
+      <c r="W19" s="14">
         <f t="shared" si="0"/>
         <v>7.3375262054507351</v>
       </c>
@@ -2354,10 +2357,10 @@
       <c r="U20" s="8">
         <v>0.50000000000000011</v>
       </c>
-      <c r="V20" s="15">
+      <c r="V20" s="14">
         <v>0.16477272727272729</v>
       </c>
-      <c r="W20" s="15">
+      <c r="W20" s="14">
         <f t="shared" si="0"/>
         <v>16.47727272727273</v>
       </c>
@@ -2445,10 +2448,10 @@
       <c r="U21" s="8">
         <v>0.49002849002849003</v>
       </c>
-      <c r="V21" s="15">
+      <c r="V21" s="14">
         <v>0.15537488708220415</v>
       </c>
-      <c r="W21" s="15">
+      <c r="W21" s="14">
         <f t="shared" si="0"/>
         <v>15.537488708220415</v>
       </c>
@@ -2536,10 +2539,10 @@
       <c r="U22" s="8">
         <v>0.49715099715099714</v>
       </c>
-      <c r="V22" s="15">
+      <c r="V22" s="14">
         <v>0.16293183940242764</v>
       </c>
-      <c r="W22" s="15">
+      <c r="W22" s="14">
         <f t="shared" si="0"/>
         <v>16.293183940242763</v>
       </c>
@@ -2627,10 +2630,10 @@
       <c r="U23" s="8">
         <v>0.47685185185185186</v>
       </c>
-      <c r="V23" s="15">
+      <c r="V23" s="14">
         <v>0.231981981981982</v>
       </c>
-      <c r="W23" s="15">
+      <c r="W23" s="14">
         <f t="shared" si="0"/>
         <v>23.198198198198199</v>
       </c>
@@ -2718,10 +2721,10 @@
       <c r="U24" s="8">
         <v>0.5131826741996236</v>
       </c>
-      <c r="V24" s="15">
+      <c r="V24" s="14">
         <v>0.23840769903762041</v>
       </c>
-      <c r="W24" s="15">
+      <c r="W24" s="14">
         <f t="shared" si="0"/>
         <v>23.840769903762041</v>
       </c>
@@ -2809,10 +2812,10 @@
       <c r="U25" s="8">
         <v>0.47743055555555569</v>
       </c>
-      <c r="V25" s="15">
+      <c r="V25" s="14">
         <v>0.20370370370370378</v>
       </c>
-      <c r="W25" s="15">
+      <c r="W25" s="14">
         <f t="shared" si="0"/>
         <v>20.370370370370377</v>
       </c>
@@ -2900,10 +2903,10 @@
       <c r="U26" s="8">
         <v>0.48148148148148145</v>
       </c>
-      <c r="V26" s="15">
+      <c r="V26" s="14">
         <v>0.25490196078431371</v>
       </c>
-      <c r="W26" s="15">
+      <c r="W26" s="14">
         <f t="shared" si="0"/>
         <v>25.490196078431371</v>
       </c>
@@ -2991,10 +2994,10 @@
       <c r="U27" s="8">
         <v>0.41798941798941813</v>
       </c>
-      <c r="V27" s="15">
+      <c r="V27" s="14">
         <v>0.10449735449735453</v>
       </c>
-      <c r="W27" s="15">
+      <c r="W27" s="14">
         <f t="shared" si="0"/>
         <v>10.449735449735453</v>
       </c>
@@ -3082,10 +3085,10 @@
       <c r="U28" s="8">
         <v>0.46180555555555564</v>
       </c>
-      <c r="V28" s="15">
+      <c r="V28" s="14">
         <v>0.17385620915032682</v>
       </c>
-      <c r="W28" s="15">
+      <c r="W28" s="14">
         <f t="shared" si="0"/>
         <v>17.385620915032682</v>
       </c>
@@ -3111,7 +3114,7 @@
     </row>
     <row r="29" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B29" s="7">
         <v>1</v>
@@ -3173,10 +3176,10 @@
       <c r="U29" s="8">
         <v>0.4982363315696649</v>
       </c>
-      <c r="V29" s="15">
+      <c r="V29" s="14">
         <v>0.33040935672514615</v>
       </c>
-      <c r="W29" s="15">
+      <c r="W29" s="14">
         <f t="shared" si="0"/>
         <v>33.040935672514614</v>
       </c>
@@ -3202,7 +3205,7 @@
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B30" s="7">
         <v>2</v>
@@ -3264,10 +3267,10 @@
       <c r="U30" s="8">
         <v>0.43888888888888894</v>
       </c>
-      <c r="V30" s="15">
+      <c r="V30" s="14">
         <v>0.23099415204678364</v>
       </c>
-      <c r="W30" s="15">
+      <c r="W30" s="14">
         <f t="shared" si="0"/>
         <v>23.099415204678365</v>
       </c>
@@ -3293,7 +3296,7 @@
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B31" s="7">
         <v>3</v>
@@ -3355,10 +3358,10 @@
       <c r="U31" s="8">
         <v>0.41975308641975317</v>
       </c>
-      <c r="V31" s="15">
+      <c r="V31" s="14">
         <v>0.13991769547325106</v>
       </c>
-      <c r="W31" s="15">
+      <c r="W31" s="14">
         <f t="shared" si="0"/>
         <v>13.991769547325106</v>
       </c>
@@ -3384,7 +3387,7 @@
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32" s="7">
         <v>4</v>
@@ -3446,10 +3449,10 @@
       <c r="U32" s="8">
         <v>0.54700854700854695</v>
       </c>
-      <c r="V32" s="15">
+      <c r="V32" s="14">
         <v>0.38647342995169082</v>
       </c>
-      <c r="W32" s="15">
+      <c r="W32" s="14">
         <f t="shared" si="0"/>
         <v>38.647342995169083</v>
       </c>
@@ -3475,7 +3478,7 @@
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B33" s="7">
         <v>5</v>
@@ -3537,10 +3540,10 @@
       <c r="U33" s="8">
         <v>0.39583333333333326</v>
       </c>
-      <c r="V33" s="15">
+      <c r="V33" s="14">
         <v>0.17592592592592587</v>
       </c>
-      <c r="W33" s="15">
+      <c r="W33" s="14">
         <f t="shared" si="0"/>
         <v>17.592592592592588</v>
       </c>
@@ -3566,7 +3569,7 @@
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B34" s="7">
         <v>6</v>
@@ -3628,10 +3631,10 @@
       <c r="U34" s="8">
         <v>0.49794238683127579</v>
       </c>
-      <c r="V34" s="15">
+      <c r="V34" s="14">
         <v>0.28009259259259262</v>
       </c>
-      <c r="W34" s="15">
+      <c r="W34" s="14">
         <f t="shared" si="0"/>
         <v>28.009259259259263</v>
       </c>
@@ -3657,7 +3660,7 @@
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" s="7">
         <v>7</v>
@@ -3719,10 +3722,10 @@
       <c r="U35" s="8">
         <v>0.45726495726495736</v>
       </c>
-      <c r="V35" s="15">
+      <c r="V35" s="14">
         <v>0.13209876543209878</v>
       </c>
-      <c r="W35" s="15">
+      <c r="W35" s="14">
         <f t="shared" si="0"/>
         <v>13.209876543209878</v>
       </c>
@@ -3748,7 +3751,7 @@
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B36" s="7">
         <v>8</v>
@@ -3810,10 +3813,10 @@
       <c r="U36" s="8">
         <v>0.39869281045751637</v>
       </c>
-      <c r="V36" s="15">
+      <c r="V36" s="14">
         <v>0.23371647509578544</v>
       </c>
-      <c r="W36" s="15">
+      <c r="W36" s="14">
         <f t="shared" si="0"/>
         <v>23.371647509578544</v>
       </c>
@@ -3839,7 +3842,7 @@
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B37" s="7">
         <v>9</v>
@@ -3901,10 +3904,10 @@
       <c r="U37" s="8">
         <v>0.43827160493827161</v>
       </c>
-      <c r="V37" s="15">
+      <c r="V37" s="14">
         <v>0.14609053497942387</v>
       </c>
-      <c r="W37" s="15">
+      <c r="W37" s="14">
         <f t="shared" si="0"/>
         <v>14.609053497942387</v>
       </c>
@@ -3930,7 +3933,7 @@
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B38" s="7">
         <v>10</v>
@@ -3992,10 +3995,10 @@
       <c r="U38" s="8">
         <v>0.35714285714285721</v>
       </c>
-      <c r="V38" s="15">
+      <c r="V38" s="14">
         <v>6.7567567567567585E-2</v>
       </c>
-      <c r="W38" s="15">
+      <c r="W38" s="14">
         <f t="shared" si="0"/>
         <v>6.7567567567567588</v>
       </c>
@@ -4021,7 +4024,7 @@
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B39" s="7">
         <v>11</v>
@@ -4083,10 +4086,10 @@
       <c r="U39" s="8">
         <v>0.47883597883597889</v>
       </c>
-      <c r="V39" s="15">
+      <c r="V39" s="14">
         <v>0.26461988304093575</v>
       </c>
-      <c r="W39" s="15">
+      <c r="W39" s="14">
         <f t="shared" si="0"/>
         <v>26.461988304093577</v>
       </c>
@@ -4112,7 +4115,7 @@
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B40" s="7">
         <v>12</v>
@@ -4174,10 +4177,10 @@
       <c r="U40" s="8">
         <v>0.47474747474747475</v>
       </c>
-      <c r="V40" s="15">
+      <c r="V40" s="14">
         <v>0.13742690058479534</v>
       </c>
-      <c r="W40" s="15">
+      <c r="W40" s="14">
         <f t="shared" si="0"/>
         <v>13.742690058479534</v>
       </c>
@@ -4203,7 +4206,7 @@
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B41" s="7">
         <v>13</v>
@@ -4265,10 +4268,10 @@
       <c r="U41" s="8">
         <v>0.54938271604938271</v>
       </c>
-      <c r="V41" s="15">
+      <c r="V41" s="14">
         <v>0.49444444444444446</v>
       </c>
-      <c r="W41" s="15">
+      <c r="W41" s="14">
         <f t="shared" si="0"/>
         <v>49.444444444444443</v>
       </c>
@@ -4294,7 +4297,7 @@
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B42" s="7">
         <v>14</v>
@@ -4356,10 +4359,10 @@
       <c r="U42" s="8">
         <v>0.49905838041431266</v>
       </c>
-      <c r="V42" s="15">
+      <c r="V42" s="14">
         <v>0.34640522875816998</v>
       </c>
-      <c r="W42" s="15">
+      <c r="W42" s="14">
         <f t="shared" si="0"/>
         <v>34.640522875816998</v>
       </c>
@@ -4447,10 +4450,10 @@
       <c r="U43" s="8">
         <v>0.33760683760683763</v>
       </c>
-      <c r="V43" s="15">
+      <c r="V43" s="14">
         <v>5.2248677248677253E-2</v>
       </c>
-      <c r="W43" s="15">
+      <c r="W43" s="14">
         <f t="shared" si="0"/>
         <v>5.2248677248677255</v>
       </c>
@@ -4538,10 +4541,10 @@
       <c r="U44" s="8">
         <v>0.38050314465408808</v>
       </c>
-      <c r="V44" s="15">
+      <c r="V44" s="14">
         <v>0.1884735202492212</v>
       </c>
-      <c r="W44" s="15">
+      <c r="W44" s="14">
         <f t="shared" si="0"/>
         <v>18.84735202492212</v>
       </c>
@@ -4629,10 +4632,10 @@
       <c r="U45" s="8">
         <v>0.47453703703703715</v>
       </c>
-      <c r="V45" s="15">
+      <c r="V45" s="14">
         <v>0.19303201506591341</v>
       </c>
-      <c r="W45" s="15">
+      <c r="W45" s="14">
         <f t="shared" si="0"/>
         <v>19.303201506591343</v>
       </c>
@@ -4720,10 +4723,10 @@
       <c r="U46" s="8">
         <v>0.48765432098765438</v>
       </c>
-      <c r="V46" s="15">
+      <c r="V46" s="14">
         <v>0.29259259259259263</v>
       </c>
-      <c r="W46" s="15">
+      <c r="W46" s="14">
         <f t="shared" si="0"/>
         <v>29.259259259259263</v>
       </c>
@@ -4811,10 +4814,10 @@
       <c r="U47" s="8">
         <v>0.4212962962962965</v>
       </c>
-      <c r="V47" s="15">
+      <c r="V47" s="14">
         <v>0.24462365591397864</v>
       </c>
-      <c r="W47" s="15">
+      <c r="W47" s="14">
         <f t="shared" si="0"/>
         <v>24.462365591397862</v>
       </c>
@@ -4902,10 +4905,10 @@
       <c r="U48" s="8">
         <v>0.43843843843843849</v>
       </c>
-      <c r="V48" s="15">
+      <c r="V48" s="14">
         <v>0.26164874551971329</v>
       </c>
-      <c r="W48" s="15">
+      <c r="W48" s="14">
         <f t="shared" si="0"/>
         <v>26.16487455197133</v>
       </c>
@@ -4931,7 +4934,7 @@
     </row>
     <row r="49" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B49" s="7">
         <v>1</v>
@@ -4993,14 +4996,14 @@
       <c r="U49" s="8">
         <v>0.36507936507936506</v>
       </c>
-      <c r="V49" s="15">
+      <c r="V49" s="14">
         <v>4.9145299145299137E-2</v>
       </c>
-      <c r="W49" s="15">
+      <c r="W49" s="14">
         <f t="shared" si="0"/>
         <v>4.9145299145299139</v>
       </c>
-      <c r="X49" s="8">
+      <c r="X49" s="14">
         <v>2.3221153846153846</v>
       </c>
       <c r="Y49" s="8">
@@ -5009,7 +5012,7 @@
       <c r="Z49" s="8">
         <v>2.8626373626373609</v>
       </c>
-      <c r="AA49" s="10">
+      <c r="AA49" s="8">
         <v>2.4579517704517708</v>
       </c>
       <c r="AB49" s="10">
@@ -5022,7 +5025,7 @@
     </row>
     <row r="50" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B50" s="7">
         <v>2</v>
@@ -5084,14 +5087,14 @@
       <c r="U50" s="8">
         <v>0.3666666666666667</v>
       </c>
-      <c r="V50" s="15">
+      <c r="V50" s="14">
         <v>6.1111111111111116E-2</v>
       </c>
-      <c r="W50" s="15">
+      <c r="W50" s="14">
         <f t="shared" si="0"/>
         <v>6.1111111111111116</v>
       </c>
-      <c r="X50" s="8">
+      <c r="X50" s="14">
         <v>2.1666666666666665</v>
       </c>
       <c r="Y50" s="8">
@@ -5100,7 +5103,7 @@
       <c r="Z50" s="8">
         <v>3.2333333333333334</v>
       </c>
-      <c r="AA50" s="10">
+      <c r="AA50" s="8">
         <v>2.5833333333333339</v>
       </c>
       <c r="AB50" s="10">
@@ -5113,7 +5116,7 @@
     </row>
     <row r="51" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B51" s="7">
         <v>3</v>
@@ -5175,14 +5178,14 @@
       <c r="U51" s="8">
         <v>0.3787878787878789</v>
       </c>
-      <c r="V51" s="15">
+      <c r="V51" s="14">
         <v>8.8652482269503577E-2</v>
       </c>
-      <c r="W51" s="15">
+      <c r="W51" s="14">
         <f t="shared" si="0"/>
         <v>8.8652482269503583</v>
       </c>
-      <c r="X51" s="8">
+      <c r="X51" s="14">
         <v>2.5053191489361701</v>
       </c>
       <c r="Y51" s="8">
@@ -5191,7 +5194,7 @@
       <c r="Z51" s="8">
         <v>3.282674772036474</v>
       </c>
-      <c r="AA51" s="10">
+      <c r="AA51" s="8">
         <v>2.9494258696386342</v>
       </c>
       <c r="AB51" s="10">
@@ -5204,31 +5207,31 @@
     </row>
     <row r="52" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B52" s="7">
         <v>4</v>
       </c>
       <c r="C52" s="8">
-        <v>2.3484848484848486</v>
+        <v>2.5681818181818183</v>
       </c>
       <c r="D52" s="8">
-        <v>1.3484848484848484</v>
+        <v>1.4772727272727273</v>
       </c>
       <c r="E52" s="8">
-        <v>2.4545454545454541</v>
+        <v>2.6161616161616164</v>
       </c>
       <c r="F52" s="8">
-        <v>1.4015151515151516</v>
+        <v>1.606060606060606</v>
       </c>
       <c r="G52" s="8">
-        <v>1.8787878787878789</v>
+        <v>2.0227272727272729</v>
       </c>
       <c r="H52" s="10">
-        <v>1.8863636363636367</v>
+        <v>2.0580808080808084</v>
       </c>
       <c r="I52" s="10">
-        <v>22.159090909090917</v>
+        <v>26.452020202020211</v>
       </c>
       <c r="J52" s="8">
         <v>0</v>
@@ -5237,65 +5240,65 @@
         <v>0</v>
       </c>
       <c r="L52" s="8">
-        <v>49.999999999999986</v>
+        <v>38.709677419354819</v>
       </c>
       <c r="M52" s="8">
         <v>0</v>
       </c>
       <c r="N52" s="8">
-        <v>16.666666666666664</v>
+        <v>12.903225806451607</v>
       </c>
       <c r="O52" s="8">
-        <v>0</v>
+        <v>12.903225806451607</v>
       </c>
       <c r="P52" s="8">
-        <v>16.666666666666664</v>
+        <v>12.903225806451607</v>
       </c>
       <c r="Q52" s="8">
         <v>0</v>
       </c>
       <c r="R52" s="8">
-        <v>16.666666666666664</v>
+        <v>12.903225806451607</v>
       </c>
       <c r="S52" s="8">
-        <v>0</v>
+        <v>9.6774193548387046</v>
       </c>
       <c r="T52" s="10">
-        <v>3.0303030303030304E-2</v>
+        <v>0.12121212121212122</v>
       </c>
       <c r="U52" s="8">
-        <v>0.33333333333333337</v>
-      </c>
-      <c r="V52" s="15">
-        <v>1.0101010101010102E-2</v>
-      </c>
-      <c r="W52" s="15">
+        <v>0.43055555555555569</v>
+      </c>
+      <c r="V52" s="14">
+        <v>5.2188552188552208E-2</v>
+      </c>
+      <c r="W52" s="14">
         <f t="shared" si="0"/>
-        <v>1.0101010101010102</v>
-      </c>
-      <c r="X52" s="8">
-        <v>2.6287878787878789</v>
+        <v>5.2188552188552206</v>
+      </c>
+      <c r="X52" s="14">
+        <v>2.8333333333333335</v>
       </c>
       <c r="Y52" s="8">
-        <v>3.2525252525252526</v>
+        <v>3.4141414141414148</v>
       </c>
       <c r="Z52" s="8">
-        <v>3.372294372294371</v>
-      </c>
-      <c r="AA52" s="10">
-        <v>3.0845358345358349</v>
+        <v>3.5844155844155847</v>
+      </c>
+      <c r="AA52" s="8">
+        <v>3.2772967772967765</v>
       </c>
       <c r="AB52" s="10">
-        <v>52.113395863395873</v>
+        <v>56.932419432419415</v>
       </c>
       <c r="AC52" s="10">
         <f t="shared" si="1"/>
-        <v>74.90580407247073</v>
+        <v>70.465568382235048</v>
       </c>
     </row>
     <row r="53" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B53" s="7">
         <v>5</v>
@@ -5357,14 +5360,14 @@
       <c r="U53" s="8">
         <v>0.35714285714285715</v>
       </c>
-      <c r="V53" s="15">
+      <c r="V53" s="14">
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="W53" s="15">
+      <c r="W53" s="14">
         <f t="shared" si="0"/>
         <v>6.666666666666667</v>
       </c>
-      <c r="X53" s="8">
+      <c r="X53" s="14">
         <v>2.8833333333333333</v>
       </c>
       <c r="Y53" s="8">
@@ -5373,7 +5376,7 @@
       <c r="Z53" s="8">
         <v>3.2761904761904774</v>
       </c>
-      <c r="AA53" s="10">
+      <c r="AA53" s="8">
         <v>3.1020634920634915</v>
       </c>
       <c r="AB53" s="10">
@@ -5386,122 +5389,122 @@
     </row>
     <row r="54" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B54" s="7">
         <v>6</v>
       </c>
       <c r="C54" s="8">
-        <v>1.3582089552238805</v>
+        <v>2.6641791044776117</v>
       </c>
       <c r="D54" s="8">
-        <v>1.3171641791044777</v>
+        <v>1.6940298507462686</v>
       </c>
       <c r="E54" s="8">
-        <v>1.5323383084577116</v>
+        <v>3.0149253731343273</v>
       </c>
       <c r="F54" s="8">
-        <v>1.0559701492537314</v>
+        <v>1.2985074626865671</v>
       </c>
       <c r="G54" s="8">
-        <v>1.7835820895522387</v>
+        <v>2.2126865671641789</v>
       </c>
       <c r="H54" s="10">
-        <v>1.4094527363184084</v>
+        <v>2.17686567164179</v>
       </c>
       <c r="I54" s="10">
-        <v>10.23631840796021</v>
+        <v>29.421641791044749</v>
       </c>
       <c r="J54" s="8">
-        <v>0</v>
+        <v>3.6144578313253009</v>
       </c>
       <c r="K54" s="8">
-        <v>0</v>
+        <v>7.2289156626506017</v>
       </c>
       <c r="L54" s="8">
-        <v>44.999999999999993</v>
+        <v>43.373493975903607</v>
       </c>
       <c r="M54" s="8">
-        <v>0</v>
+        <v>7.2289156626506017</v>
       </c>
       <c r="N54" s="8">
-        <v>14.999999999999996</v>
+        <v>9.6385542168674672</v>
       </c>
       <c r="O54" s="8">
-        <v>9.9999999999999982</v>
+        <v>2.4096385542168668</v>
       </c>
       <c r="P54" s="8">
-        <v>4.9999999999999991</v>
+        <v>7.2289156626506008</v>
       </c>
       <c r="Q54" s="8">
         <v>0</v>
       </c>
       <c r="R54" s="8">
-        <v>14.999999999999996</v>
+        <v>14.457831325301202</v>
       </c>
       <c r="S54" s="8">
-        <v>9.9999999999999982</v>
+        <v>4.8192771084337336</v>
       </c>
       <c r="T54" s="10">
-        <v>4.4776119402985072E-2</v>
+        <v>0.17910447761194029</v>
       </c>
       <c r="U54" s="8">
-        <v>0.37037037037037041</v>
-      </c>
-      <c r="V54" s="15">
-        <v>1.658374792703151E-2</v>
-      </c>
-      <c r="W54" s="15">
+        <v>0.3842592592592593</v>
+      </c>
+      <c r="V54" s="14">
+        <v>6.8822553897180769E-2</v>
+      </c>
+      <c r="W54" s="14">
         <f t="shared" si="0"/>
-        <v>1.6583747927031509</v>
-      </c>
-      <c r="X54" s="8">
-        <v>1.6455223880597014</v>
+        <v>6.8822553897180772</v>
+      </c>
+      <c r="X54" s="14">
+        <v>2.5</v>
       </c>
       <c r="Y54" s="8">
-        <v>2.6169154228855729</v>
+        <v>2.5796019900497513</v>
       </c>
       <c r="Z54" s="8">
-        <v>2.4605543710021318</v>
-      </c>
-      <c r="AA54" s="10">
-        <v>2.2409973939824686</v>
+        <v>2.8443496801705757</v>
+      </c>
+      <c r="AA54" s="8">
+        <v>2.6413172234067748</v>
       </c>
       <c r="AB54" s="10">
-        <v>31.024934849561713</v>
+        <v>41.032930585169368</v>
       </c>
       <c r="AC54" s="10">
         <f t="shared" si="1"/>
-        <v>85.693457316591648</v>
+        <v>74.221057411355943</v>
       </c>
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B55" s="7">
         <v>7</v>
       </c>
       <c r="C55" s="8">
-        <v>1.4375</v>
+        <v>3.1590909090909092</v>
       </c>
       <c r="D55" s="8">
-        <v>1.2840909090909092</v>
+        <v>1.9375</v>
       </c>
       <c r="E55" s="8">
-        <v>1.4772727272727273</v>
+        <v>3.3181818181818183</v>
       </c>
       <c r="F55" s="8">
-        <v>1.0625</v>
+        <v>1.1875</v>
       </c>
       <c r="G55" s="8">
-        <v>2.1136363636363638</v>
+        <v>2.7272727272727271</v>
       </c>
       <c r="H55" s="10">
-        <v>1.4750000000000012</v>
+        <v>2.4659090909090904</v>
       </c>
       <c r="I55" s="10">
-        <v>11.87500000000003</v>
+        <v>36.647727272727259</v>
       </c>
       <c r="J55" s="8">
         <v>0</v>
@@ -5510,60 +5513,60 @@
         <v>0</v>
       </c>
       <c r="L55" s="8">
-        <v>49.999999999999993</v>
+        <v>40</v>
       </c>
       <c r="M55" s="8">
-        <v>0</v>
+        <v>29.999999999999993</v>
       </c>
       <c r="N55" s="8">
-        <v>16.666666666666664</v>
+        <v>11.666666666666666</v>
       </c>
       <c r="O55" s="8">
         <v>0</v>
       </c>
       <c r="P55" s="8">
-        <v>0</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="Q55" s="8">
         <v>0</v>
       </c>
       <c r="R55" s="8">
-        <v>16.666666666666664</v>
+        <v>13.333333333333334</v>
       </c>
       <c r="S55" s="8">
-        <v>16.666666666666664</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="T55" s="10">
-        <v>2.2727272727272728E-2</v>
+        <v>0.18181818181818182</v>
       </c>
       <c r="U55" s="8">
-        <v>0.33333333333333337</v>
-      </c>
-      <c r="V55" s="15">
-        <v>7.5757575757575768E-3</v>
-      </c>
-      <c r="W55" s="15">
+        <v>0.41666666666666663</v>
+      </c>
+      <c r="V55" s="14">
+        <v>7.575757575757576E-2</v>
+      </c>
+      <c r="W55" s="14">
         <f t="shared" si="0"/>
-        <v>0.75757575757575768</v>
-      </c>
-      <c r="X55" s="8">
-        <v>1.3863636363636365</v>
+        <v>7.5757575757575761</v>
+      </c>
+      <c r="X55" s="14">
+        <v>2.4034090909090908</v>
       </c>
       <c r="Y55" s="8">
-        <v>2.4999999999999996</v>
+        <v>2.1515151515151518</v>
       </c>
       <c r="Z55" s="8">
-        <v>2.2370129870129869</v>
-      </c>
-      <c r="AA55" s="10">
-        <v>2.0411255411255413</v>
+        <v>2.8733766233766231</v>
+      </c>
+      <c r="AA55" s="8">
+        <v>2.4761002886002883</v>
       </c>
       <c r="AB55" s="10">
-        <v>26.028138528138534</v>
+        <v>36.902507215007205</v>
       </c>
       <c r="AC55" s="10">
         <f t="shared" si="1"/>
-        <v>87.113095238095227</v>
+        <v>72.958002645502646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>